<commit_message>
Initial commit - SeniorCare project
</commit_message>
<xml_diff>
--- a/sample_data.xlsx
+++ b/sample_data.xlsx
@@ -407,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -496,24 +496,24 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>caretaker.test@seniorcare.local</v>
+        <v>family2.test@seniorcare.local</v>
       </c>
       <c r="B6" t="str">
-        <v>Anitha Krishnan</v>
+        <v>Vignesh Ramesh</v>
       </c>
       <c r="C6" t="str">
-        <v>caretaker</v>
+        <v>family_member</v>
       </c>
       <c r="D6" t="str">
-        <v>+91 98765 00004</v>
+        <v>+91 98765 00006</v>
       </c>
       <c r="E6" t="str">
-        <v>Mylapore, Chennai</v>
+        <v>Adyar, Chennai</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>caregiver.test@seniorcare.local</v>
+        <v>caretaker.test@seniorcare.local</v>
       </c>
       <c r="B7" t="str">
         <v>Anitha Krishnan</v>
@@ -530,24 +530,58 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>caregiver.test@seniorcare.local</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Anitha Krishnan</v>
+      </c>
+      <c r="C8" t="str">
+        <v>caretaker</v>
+      </c>
+      <c r="D8" t="str">
+        <v>+91 98765 00004</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Mylapore, Chennai</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>volunteer.test@seniorcare.local</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B9" t="str">
         <v>Karthik Raman</v>
       </c>
-      <c r="C8" t="str">
+      <c r="C9" t="str">
         <v>volunteer</v>
       </c>
-      <c r="D8" t="str">
+      <c r="D9" t="str">
         <v>+91 98765 00005</v>
       </c>
-      <c r="E8" t="str">
+      <c r="E9" t="str">
         <v>Thiruvanmiyur, Chennai</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>temp.caregiver@seniorcare.local</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Dinesh Kumar (Probation)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>caretaker</v>
+      </c>
+      <c r="D10" t="str">
+        <v>+91 98765 00099</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Tambaram, Chennai</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1151,7 +1185,7 @@
         <v>Feeling great today, completed morning walk.</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-10-04T17:06:13.611Z</v>
+        <v>2026-10-05T15:17:46.973Z</v>
       </c>
     </row>
     <row r="3">
@@ -1168,7 +1202,7 @@
         <v>Took morning medications on time.</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-10-03T17:06:13.611Z</v>
+        <v>2026-10-04T15:17:46.973Z</v>
       </c>
     </row>
     <row r="4">
@@ -1185,7 +1219,7 @@
         <v>Slight joint ache, applied ointment.</v>
       </c>
       <c r="E4" t="str">
-        <v>2026-10-02T17:06:13.611Z</v>
+        <v>2026-10-03T15:17:46.973Z</v>
       </c>
     </row>
     <row r="5">
@@ -1202,7 +1236,7 @@
         <v>Physiotherapy exercises done.</v>
       </c>
       <c r="E5" t="str">
-        <v>2026-10-04T17:06:13.611Z</v>
+        <v>2026-10-05T15:17:46.973Z</v>
       </c>
     </row>
     <row r="6">
@@ -1219,7 +1253,7 @@
         <v>All good, had breakfast.</v>
       </c>
       <c r="E6" t="str">
-        <v>2026-10-04T17:06:13.611Z</v>
+        <v>2026-10-05T15:17:46.973Z</v>
       </c>
     </row>
     <row r="7">
@@ -1236,7 +1270,7 @@
         <v>Resting comfortably.</v>
       </c>
       <c r="E7" t="str">
-        <v>2026-10-03T17:06:13.611Z</v>
+        <v>2026-10-04T15:17:46.973Z</v>
       </c>
     </row>
   </sheetData>
@@ -1361,7 +1395,7 @@
         <v>Apollo Senior Health Center</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-10-05 10:30 AM</v>
+        <v>2026-10-06 10:30 AM</v>
       </c>
       <c r="G2" t="str">
         <v>Upcoming</v>
@@ -1384,7 +1418,7 @@
         <v>Sankara Nethralaya</v>
       </c>
       <c r="F3" t="str">
-        <v>2026-10-07 02:00 PM</v>
+        <v>2026-10-08 02:00 PM</v>
       </c>
       <c r="G3" t="str">
         <v>Upcoming</v>
@@ -1407,7 +1441,7 @@
         <v>Fortis Malar Hospital</v>
       </c>
       <c r="F4" t="str">
-        <v>2026-10-09 11:15 AM</v>
+        <v>2026-10-10 11:15 AM</v>
       </c>
       <c r="G4" t="str">
         <v>Upcoming</v>
@@ -1430,7 +1464,7 @@
         <v>Apollo Senior Health Center</v>
       </c>
       <c r="F5" t="str">
-        <v>2026-09-27 09:30 AM</v>
+        <v>2026-09-28 09:30 AM</v>
       </c>
       <c r="G5" t="str">
         <v>Completed</v>

</xml_diff>